<commit_message>
Update Patient Inbox Email Test Plan document to reflect recent changes
</commit_message>
<xml_diff>
--- a/docs/US42595_Patient_Inbox_Email_Multiple_Items_Test_Plan_AC_Traceability.xlsx
+++ b/docs/US42595_Patient_Inbox_Email_Multiple_Items_Test_Plan_AC_Traceability.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://fidelitylifenz-my.sharepoint.com/personal/deepika_udesh_fidelitylife_co_nz/Documents/Desktop/NotepadProject/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="8_{C2FB42C4-CAD5-4EC6-8FCC-E4D329301FD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CB95035B-7F54-426C-AB38-3A609B514C08}"/>
+  <xr:revisionPtr revIDLastSave="67" documentId="8_{C2FB42C4-CAD5-4EC6-8FCC-E4D329301FD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CEF4C77F-334B-451D-B34C-896186627017}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,7 @@
     <sheet name="Risk Areas" sheetId="4" r:id="rId4"/>
     <sheet name="Test Data" sheetId="5" r:id="rId5"/>
     <sheet name="Out of Scope" sheetId="6" r:id="rId6"/>
+    <sheet name="Defect Report" sheetId="7" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Cases'!$A$1:$K$17</definedName>
@@ -47,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="281">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="414" uniqueCount="298">
   <si>
     <t>Manual Test Plan - User Story 42595: Patient Inbox Email Multiple Items</t>
   </si>
@@ -925,12 +926,182 @@
   <si>
     <t>Covered by wider security regression if impacted.</t>
   </si>
+  <si>
+    <t xml:space="preserve">Title: </t>
+  </si>
+  <si>
+    <t>UAT-Email Patient button is not displayed in Patient Inbox Toolbar</t>
+  </si>
+  <si>
+    <t>Description:</t>
+  </si>
+  <si>
+    <t>The Email Patient button is not displayed in the Others section of the Patient Inbox toolbar. The Email Recipient button is visible, but the Email Patient button is missing.</t>
+  </si>
+  <si>
+    <t>Repro Steps:</t>
+  </si>
+  <si>
+    <t>Actual Result:</t>
+  </si>
+  <si>
+    <t>Expected Result:</t>
+  </si>
+  <si>
+    <t>Only Email Recipient is displayed.
+Email Patient button is missing from the toolbar.</t>
+  </si>
+  <si>
+    <t>Both Email Patient and Email Recipient buttons are displayed in the Others section of the Patient Inbox toolbar</t>
+  </si>
+  <si>
+    <t>Severity:</t>
+  </si>
+  <si>
+    <t>Priority:</t>
+  </si>
+  <si>
+    <t>UserStory:</t>
+  </si>
+  <si>
+    <t>TestCase:</t>
+  </si>
+  <si>
+    <t>S3</t>
+  </si>
+  <si>
+    <t>42595 - Patient Inbox: Email Multiple Items</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">PreConditions: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+-User has access to Patient Inbox.
+-Patient record contains Patient Inbox items.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Steps:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">- Open a patient record.
+- Navigate to Patient Tab &gt; Patient Inbox.
+- Locate the Others section on the toolbar.
+- Review the available actions.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>AC Impacted:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+AC01
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Business Impact:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Users cannot email multiple Patient Inbox items directly to the patient from the Patient Inbox toolbar, preventing use of a key feature delivered by User Story 42595
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Evidence:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Screenshot of Patient Inbox toolbar.
+Screenshot showing missing Email Patient button.</t>
+    </r>
+  </si>
+  <si>
+    <t>Sample Defect Report</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -980,8 +1151,16 @@
       <color rgb="FF1F4E78"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1012,6 +1191,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1139,20 +1330,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -1195,6 +1375,29 @@
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1205,42 +1408,6 @@
         <left style="thin">
           <color indexed="64"/>
         </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
         <right/>
         <top style="thin">
           <color indexed="64"/>
@@ -1299,10 +1466,21 @@
       </border>
     </dxf>
     <dxf>
-      <border>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
       </border>
     </dxf>
     <dxf>
@@ -1322,21 +1500,10 @@
       </border>
     </dxf>
     <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
+      <border>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
       </border>
     </dxf>
     <dxf>
@@ -1464,10 +1631,21 @@
       </border>
     </dxf>
     <dxf>
-      <border>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
       </border>
     </dxf>
     <dxf>
@@ -1487,21 +1665,10 @@
       </border>
     </dxf>
     <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
+      <border>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
       </border>
     </dxf>
     <dxf>
@@ -1629,6 +1796,40 @@
       </border>
     </dxf>
     <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
       <border>
         <bottom style="thin">
           <color indexed="64"/>
@@ -1643,9 +1844,128 @@
         <right style="thin">
           <color indexed="64"/>
         </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
         <top style="thin">
           <color indexed="64"/>
         </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
@@ -1661,123 +1981,6 @@
         </right>
         <top/>
         <bottom/>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
         <vertical style="thin">
           <color indexed="64"/>
         </vertical>
@@ -1800,54 +2003,54 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="ACTraceabilityTable" displayName="ACTraceabilityTable" ref="A1:E24" headerRowDxfId="25" headerRowBorderDxfId="26">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="ACTraceabilityTable" displayName="ACTraceabilityTable" ref="A1:E24" headerRowDxfId="31" headerRowBorderDxfId="30">
   <autoFilter ref="A1:E24" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="AC ID" dataDxfId="31"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Acceptance Criteria" dataDxfId="30"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Mapped Test Cases" dataDxfId="29"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Coverage Status" dataDxfId="28"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Coverage Notes" dataDxfId="27"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="AC ID" dataDxfId="29"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Acceptance Criteria" dataDxfId="28"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Mapped Test Cases" dataDxfId="27"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Coverage Status" dataDxfId="26"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Coverage Notes" dataDxfId="25"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="RiskAreasTable" displayName="RiskAreasTable" ref="A1:E4" headerRowDxfId="17" totalsRowDxfId="16" headerRowBorderDxfId="23" tableBorderDxfId="24">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="RiskAreasTable" displayName="RiskAreasTable" ref="A1:E4" headerRowDxfId="24" totalsRowDxfId="21" headerRowBorderDxfId="23" tableBorderDxfId="22">
   <autoFilter ref="A1:E4" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="Risk ID" dataDxfId="22"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Risk Area" dataDxfId="21"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Why it is high risk" dataDxfId="20"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="Clinical priority / impact" dataDxfId="19"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="Mitigation in test plan" dataDxfId="18"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="Risk ID" dataDxfId="20"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Risk Area" dataDxfId="19"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Why it is high risk" dataDxfId="18"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="Clinical priority / impact" dataDxfId="17"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="Mitigation in test plan" dataDxfId="16"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="TestDataTable" displayName="TestDataTable" ref="A1:E8" headerRowDxfId="8" totalsRowDxfId="7" headerRowBorderDxfId="14" tableBorderDxfId="15">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="TestDataTable" displayName="TestDataTable" ref="A1:E8" headerRowDxfId="15" totalsRowDxfId="12" headerRowBorderDxfId="14" tableBorderDxfId="13">
   <autoFilter ref="A1:E8" xr:uid="{00000000-0009-0000-0100-000003000000}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="Data ID" dataDxfId="13"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="Data Needed" dataDxfId="12"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="Purpose" dataDxfId="11"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0200-000004000000}" name="Safe clinical test data approach" dataDxfId="10"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0200-000005000000}" name="Example / Notes" dataDxfId="9"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="Data ID" dataDxfId="11"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="Data Needed" dataDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="Purpose" dataDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0200-000004000000}" name="Safe clinical test data approach" dataDxfId="8"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0200-000005000000}" name="Example / Notes" dataDxfId="7"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="OutofScopeTable" displayName="OutofScopeTable" ref="A1:C6" headerRowDxfId="1" totalsRowDxfId="0" headerRowBorderDxfId="5" tableBorderDxfId="6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="OutofScopeTable" displayName="OutofScopeTable" ref="A1:C6" headerRowDxfId="6" totalsRowDxfId="3" headerRowBorderDxfId="5" tableBorderDxfId="4">
   <autoFilter ref="A1:C6" xr:uid="{00000000-0009-0000-0100-000004000000}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="Item" dataDxfId="4"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="Out of scope decision" dataDxfId="3"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="Reason" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="Item" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="Out of scope decision" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="Reason" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2150,81 +2353,81 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
+      <c r="G2" s="17"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="5"/>
-      <c r="D3" s="5"/>
-      <c r="E3" s="5"/>
-      <c r="F3" s="5"/>
-      <c r="G3" s="5"/>
+      <c r="C3" s="17"/>
+      <c r="D3" s="17"/>
+      <c r="E3" s="17"/>
+      <c r="F3" s="17"/>
+      <c r="G3" s="17"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5"/>
-      <c r="G4" s="5"/>
+      <c r="C4" s="17"/>
+      <c r="D4" s="17"/>
+      <c r="E4" s="17"/>
+      <c r="F4" s="17"/>
+      <c r="G4" s="17"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="C5" s="5"/>
-      <c r="D5" s="5"/>
-      <c r="E5" s="5"/>
-      <c r="F5" s="5"/>
-      <c r="G5" s="5"/>
+      <c r="C5" s="17"/>
+      <c r="D5" s="17"/>
+      <c r="E5" s="17"/>
+      <c r="F5" s="17"/>
+      <c r="G5" s="17"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="6" t="str">
+      <c r="B6" s="20" t="str">
         <f>COUNTIF('AC Traceability'!D:D,"Covered")&amp;" of "&amp;COUNTA('AC Traceability'!A:A)-1&amp;" covered"</f>
         <v>23 of 23 covered</v>
       </c>
-      <c r="C6" s="5"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="5"/>
-      <c r="F6" s="5"/>
-      <c r="G6" s="5"/>
+      <c r="C6" s="17"/>
+      <c r="D6" s="17"/>
+      <c r="E6" s="17"/>
+      <c r="F6" s="17"/>
+      <c r="G6" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -2261,597 +2464,597 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="B1" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="C1" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="D1" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="E1" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="F1" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="G1" s="9" t="s">
+      <c r="G1" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="H1" s="9" t="s">
+      <c r="H1" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="I1" s="9" t="s">
+      <c r="I1" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="J1" s="9" t="s">
+      <c r="J1" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="K1" s="9" t="s">
+      <c r="K1" s="4" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="87.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="C2" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="D2" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="E2" s="7" t="s">
+      <c r="E2" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="F2" s="7" t="s">
+      <c r="F2" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="G2" s="19" t="s">
+      <c r="G2" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="H2" s="7" t="s">
+      <c r="H2" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="I2" s="7" t="s">
+      <c r="I2" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="J2" s="8" t="s">
+      <c r="J2" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="K2" s="7" t="s">
+      <c r="K2" s="2" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="87.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="D3" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="F3" s="7" t="s">
+      <c r="F3" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="G3" s="19" t="s">
+      <c r="G3" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="H3" s="7" t="s">
+      <c r="H3" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="I3" s="7" t="s">
+      <c r="I3" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="J3" s="8" t="s">
+      <c r="J3" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="K3" s="7" t="s">
+      <c r="K3" s="2" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="87.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="D4" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="E4" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="F4" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="G4" s="19" t="s">
+      <c r="G4" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="H4" s="7" t="s">
+      <c r="H4" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="I4" s="7" t="s">
+      <c r="I4" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="J4" s="8" t="s">
+      <c r="J4" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="K4" s="7" t="s">
+      <c r="K4" s="2" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="87.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="7" t="s">
+      <c r="A5" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="D5" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="E5" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="F5" s="7" t="s">
+      <c r="F5" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="G5" s="19" t="s">
+      <c r="G5" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="H5" s="7" t="s">
+      <c r="H5" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="I5" s="7" t="s">
+      <c r="I5" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="J5" s="8" t="s">
+      <c r="J5" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="K5" s="7" t="s">
+      <c r="K5" s="2" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="87.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="7" t="s">
+      <c r="A6" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="E6" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="F6" s="7" t="s">
+      <c r="F6" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="G6" s="19" t="s">
+      <c r="G6" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="H6" s="7" t="s">
+      <c r="H6" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="I6" s="7" t="s">
+      <c r="I6" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="J6" s="8" t="s">
+      <c r="J6" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="K6" s="7" t="s">
+      <c r="K6" s="2" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="87.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="7" t="s">
+      <c r="A7" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="D7" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="E7" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="F7" s="7" t="s">
+      <c r="F7" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="G7" s="19" t="s">
+      <c r="G7" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="H7" s="7" t="s">
+      <c r="H7" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="I7" s="7" t="s">
+      <c r="I7" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="J7" s="8" t="s">
+      <c r="J7" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="K7" s="7" t="s">
+      <c r="K7" s="2" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="87.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="7" t="s">
+      <c r="A8" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="E8" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="F8" s="7" t="s">
+      <c r="F8" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="G8" s="19" t="s">
+      <c r="G8" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="H8" s="7" t="s">
+      <c r="H8" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="I8" s="7" t="s">
+      <c r="I8" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="J8" s="8" t="s">
+      <c r="J8" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="K8" s="7" t="s">
+      <c r="K8" s="2" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="87.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="7" t="s">
+      <c r="A9" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="C9" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="D9" s="7" t="s">
+      <c r="D9" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="E9" s="7" t="s">
+      <c r="E9" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="F9" s="7" t="s">
+      <c r="F9" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="G9" s="19" t="s">
+      <c r="G9" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="H9" s="7" t="s">
+      <c r="H9" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="I9" s="7" t="s">
+      <c r="I9" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="J9" s="8" t="s">
+      <c r="J9" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="K9" s="7" t="s">
+      <c r="K9" s="2" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="10" spans="1:11" ht="87.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="7" t="s">
+      <c r="A10" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="C10" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="D10" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="E10" s="7" t="s">
+      <c r="E10" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="F10" s="7" t="s">
+      <c r="F10" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="G10" s="19" t="s">
+      <c r="G10" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="H10" s="7" t="s">
+      <c r="H10" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="I10" s="7" t="s">
+      <c r="I10" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="J10" s="8" t="s">
+      <c r="J10" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="K10" s="7" t="s">
+      <c r="K10" s="2" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="11" spans="1:11" ht="87.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="7" t="s">
+      <c r="A11" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="C11" s="7" t="s">
+      <c r="C11" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="D11" s="7" t="s">
+      <c r="D11" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="E11" s="7" t="s">
+      <c r="E11" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="F11" s="7" t="s">
+      <c r="F11" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="G11" s="19" t="s">
+      <c r="G11" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="H11" s="7" t="s">
+      <c r="H11" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="I11" s="7" t="s">
+      <c r="I11" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="J11" s="8" t="s">
+      <c r="J11" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="K11" s="7" t="s">
+      <c r="K11" s="2" t="s">
         <v>102</v>
       </c>
     </row>
     <row r="12" spans="1:11" ht="87.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="7" t="s">
+      <c r="A12" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="B12" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="C12" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="D12" s="7" t="s">
+      <c r="D12" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="E12" s="7" t="s">
+      <c r="E12" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="F12" s="7" t="s">
+      <c r="F12" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="G12" s="19" t="s">
+      <c r="G12" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="H12" s="7" t="s">
+      <c r="H12" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="I12" s="7" t="s">
+      <c r="I12" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="J12" s="8" t="s">
+      <c r="J12" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="K12" s="7" t="s">
+      <c r="K12" s="2" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="13" spans="1:11" ht="87.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="7" t="s">
+      <c r="A13" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="B13" s="7" t="s">
+      <c r="B13" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="C13" s="7" t="s">
+      <c r="C13" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="D13" s="7" t="s">
+      <c r="D13" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="E13" s="7" t="s">
+      <c r="E13" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="F13" s="7" t="s">
+      <c r="F13" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="G13" s="19" t="s">
+      <c r="G13" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="H13" s="7" t="s">
+      <c r="H13" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="I13" s="7" t="s">
+      <c r="I13" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="J13" s="8" t="s">
+      <c r="J13" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="K13" s="7" t="s">
+      <c r="K13" s="2" t="s">
         <v>119</v>
       </c>
     </row>
     <row r="14" spans="1:11" ht="87.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="7" t="s">
+      <c r="A14" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="B14" s="7" t="s">
+      <c r="B14" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="C14" s="7" t="s">
+      <c r="C14" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="D14" s="7" t="s">
+      <c r="D14" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="E14" s="7" t="s">
+      <c r="E14" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="F14" s="7" t="s">
+      <c r="F14" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="G14" s="20" t="s">
+      <c r="G14" s="15" t="s">
         <v>126</v>
       </c>
-      <c r="H14" s="7" t="s">
+      <c r="H14" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="I14" s="7" t="s">
+      <c r="I14" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="J14" s="8" t="s">
+      <c r="J14" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="K14" s="7" t="s">
+      <c r="K14" s="2" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="15" spans="1:11" ht="87.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="7" t="s">
+      <c r="A15" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="B15" s="7" t="s">
+      <c r="B15" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="C15" s="7" t="s">
+      <c r="C15" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="D15" s="7" t="s">
+      <c r="D15" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="E15" s="7" t="s">
+      <c r="E15" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="F15" s="7" t="s">
+      <c r="F15" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="G15" s="20" t="s">
+      <c r="G15" s="15" t="s">
         <v>126</v>
       </c>
-      <c r="H15" s="7" t="s">
+      <c r="H15" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="I15" s="7" t="s">
+      <c r="I15" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="J15" s="8" t="s">
+      <c r="J15" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="K15" s="7" t="s">
+      <c r="K15" s="2" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="16" spans="1:11" ht="87.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="7" t="s">
+      <c r="A16" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="B16" s="7" t="s">
+      <c r="B16" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="C16" s="7" t="s">
+      <c r="C16" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="D16" s="7" t="s">
+      <c r="D16" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="E16" s="7" t="s">
+      <c r="E16" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="F16" s="7" t="s">
+      <c r="F16" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="G16" s="20" t="s">
+      <c r="G16" s="15" t="s">
         <v>126</v>
       </c>
-      <c r="H16" s="7" t="s">
+      <c r="H16" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="I16" s="7" t="s">
+      <c r="I16" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="J16" s="8" t="s">
+      <c r="J16" s="3" t="s">
         <v>144</v>
       </c>
-      <c r="K16" s="7" t="s">
+      <c r="K16" s="2" t="s">
         <v>145</v>
       </c>
     </row>
     <row r="17" spans="1:11" ht="87.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="7" t="s">
+      <c r="A17" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="B17" s="7" t="s">
+      <c r="B17" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="C17" s="7" t="s">
+      <c r="C17" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="D17" s="7" t="s">
+      <c r="D17" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="E17" s="7" t="s">
+      <c r="E17" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="F17" s="7" t="s">
+      <c r="F17" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="G17" s="19" t="s">
+      <c r="G17" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="H17" s="7" t="s">
+      <c r="H17" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="I17" s="7" t="s">
+      <c r="I17" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="J17" s="8" t="s">
+      <c r="J17" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="K17" s="7" t="s">
+      <c r="K17" s="2" t="s">
         <v>152</v>
       </c>
     </row>
@@ -2883,410 +3086,410 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="4" t="s">
         <v>153</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="B1" s="4" t="s">
         <v>154</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="C1" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="D1" s="4" t="s">
         <v>156</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="E1" s="4" t="s">
         <v>157</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="2" t="s">
         <v>158</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="C2" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D2" s="10" t="s">
+      <c r="D2" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="E2" s="7" t="s">
+      <c r="E2" s="2" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="D3" s="10" t="s">
+      <c r="D3" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="2" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="2" t="s">
         <v>164</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="D4" s="10" t="s">
+      <c r="D4" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="E4" s="2" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="7" t="s">
+      <c r="A5" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="D5" s="10" t="s">
+      <c r="D5" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="E5" s="2" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="7" t="s">
+      <c r="A6" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="2" t="s">
         <v>167</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="D6" s="10" t="s">
+      <c r="D6" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="E6" s="2" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="7" t="s">
+      <c r="A7" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="D7" s="10" t="s">
+      <c r="D7" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="E7" s="2" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="7" t="s">
+      <c r="A8" s="2" t="s">
         <v>169</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="2" t="s">
         <v>170</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="D8" s="10" t="s">
+      <c r="D8" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="E8" s="2" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="7" t="s">
+      <c r="A9" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="2" t="s">
         <v>172</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="C9" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="D9" s="10" t="s">
+      <c r="D9" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="E9" s="7" t="s">
+      <c r="E9" s="2" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="7" t="s">
+      <c r="A10" s="2" t="s">
         <v>173</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="2" t="s">
         <v>174</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="C10" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="D10" s="10" t="s">
+      <c r="D10" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="E10" s="7" t="s">
+      <c r="E10" s="2" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="7" t="s">
+      <c r="A11" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="2" t="s">
         <v>176</v>
       </c>
-      <c r="C11" s="7" t="s">
+      <c r="C11" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="D11" s="10" t="s">
+      <c r="D11" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="E11" s="7" t="s">
+      <c r="E11" s="2" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="7" t="s">
+      <c r="A12" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="B12" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="C12" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="D12" s="10" t="s">
+      <c r="D12" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="E12" s="7" t="s">
+      <c r="E12" s="2" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="7" t="s">
+      <c r="A13" s="2" t="s">
         <v>180</v>
       </c>
-      <c r="B13" s="7" t="s">
+      <c r="B13" s="2" t="s">
         <v>181</v>
       </c>
-      <c r="C13" s="7" t="s">
+      <c r="C13" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="D13" s="10" t="s">
+      <c r="D13" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="E13" s="7" t="s">
+      <c r="E13" s="2" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="7" t="s">
+      <c r="A14" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="B14" s="7" t="s">
+      <c r="B14" s="2" t="s">
         <v>182</v>
       </c>
-      <c r="C14" s="7" t="s">
+      <c r="C14" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="D14" s="10" t="s">
+      <c r="D14" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="E14" s="7" t="s">
+      <c r="E14" s="2" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="7" t="s">
+      <c r="A15" s="2" t="s">
         <v>183</v>
       </c>
-      <c r="B15" s="7" t="s">
+      <c r="B15" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="C15" s="7" t="s">
+      <c r="C15" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="D15" s="10" t="s">
+      <c r="D15" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="E15" s="7" t="s">
+      <c r="E15" s="2" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="7" t="s">
+      <c r="A16" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="B16" s="7" t="s">
+      <c r="B16" s="2" t="s">
         <v>186</v>
       </c>
-      <c r="C16" s="7" t="s">
+      <c r="C16" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="D16" s="10" t="s">
+      <c r="D16" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="E16" s="7" t="s">
+      <c r="E16" s="2" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="7" t="s">
+      <c r="A17" s="2" t="s">
         <v>187</v>
       </c>
-      <c r="B17" s="7" t="s">
+      <c r="B17" s="2" t="s">
         <v>188</v>
       </c>
-      <c r="C17" s="7" t="s">
+      <c r="C17" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="D17" s="10" t="s">
+      <c r="D17" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="E17" s="7" t="s">
+      <c r="E17" s="2" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="7" t="s">
+      <c r="A18" s="2" t="s">
         <v>189</v>
       </c>
-      <c r="B18" s="7" t="s">
+      <c r="B18" s="2" t="s">
         <v>190</v>
       </c>
-      <c r="C18" s="7" t="s">
+      <c r="C18" s="2" t="s">
         <v>191</v>
       </c>
-      <c r="D18" s="10" t="s">
+      <c r="D18" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="E18" s="7" t="s">
+      <c r="E18" s="2" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="7" t="s">
+      <c r="A19" s="2" t="s">
         <v>151</v>
       </c>
-      <c r="B19" s="7" t="s">
+      <c r="B19" s="2" t="s">
         <v>192</v>
       </c>
-      <c r="C19" s="7" t="s">
+      <c r="C19" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="D19" s="10" t="s">
+      <c r="D19" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="E19" s="7" t="s">
+      <c r="E19" s="2" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="7" t="s">
+      <c r="A20" s="2" t="s">
         <v>193</v>
       </c>
-      <c r="B20" s="7" t="s">
+      <c r="B20" s="2" t="s">
         <v>194</v>
       </c>
-      <c r="C20" s="7" t="s">
+      <c r="C20" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="D20" s="10" t="s">
+      <c r="D20" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="E20" s="7" t="s">
+      <c r="E20" s="2" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="7" t="s">
+      <c r="A21" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="B21" s="7" t="s">
+      <c r="B21" s="2" t="s">
         <v>196</v>
       </c>
-      <c r="C21" s="7" t="s">
+      <c r="C21" s="2" t="s">
         <v>197</v>
       </c>
-      <c r="D21" s="10" t="s">
+      <c r="D21" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="E21" s="7" t="s">
+      <c r="E21" s="2" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="7" t="s">
+      <c r="A22" s="2" t="s">
         <v>198</v>
       </c>
-      <c r="B22" s="7" t="s">
+      <c r="B22" s="2" t="s">
         <v>199</v>
       </c>
-      <c r="C22" s="7" t="s">
+      <c r="C22" s="2" t="s">
         <v>197</v>
       </c>
-      <c r="D22" s="10" t="s">
+      <c r="D22" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="E22" s="7" t="s">
+      <c r="E22" s="2" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="7" t="s">
+      <c r="A23" s="2" t="s">
         <v>200</v>
       </c>
-      <c r="B23" s="7" t="s">
+      <c r="B23" s="2" t="s">
         <v>201</v>
       </c>
-      <c r="C23" s="7" t="s">
+      <c r="C23" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="D23" s="10" t="s">
+      <c r="D23" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="E23" s="7" t="s">
+      <c r="E23" s="2" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="7" t="s">
+      <c r="A24" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="B24" s="7" t="s">
+      <c r="B24" s="2" t="s">
         <v>202</v>
       </c>
-      <c r="C24" s="7" t="s">
+      <c r="C24" s="2" t="s">
         <v>203</v>
       </c>
-      <c r="D24" s="10" t="s">
+      <c r="D24" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="E24" s="7" t="s">
+      <c r="E24" s="2" t="s">
         <v>161</v>
       </c>
     </row>
@@ -3315,70 +3518,70 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="6" t="s">
         <v>204</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="7" t="s">
         <v>205</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" s="7" t="s">
         <v>206</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="D1" s="7" t="s">
         <v>207</v>
       </c>
-      <c r="E1" s="13" t="s">
+      <c r="E1" s="8" t="s">
         <v>208</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="9" t="s">
         <v>209</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="2" t="s">
         <v>210</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="C2" s="2" t="s">
         <v>211</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="D2" s="2" t="s">
         <v>212</v>
       </c>
-      <c r="E2" s="15" t="s">
+      <c r="E2" s="10" t="s">
         <v>213</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A3" s="14" t="s">
+      <c r="A3" s="9" t="s">
         <v>214</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="2" t="s">
         <v>215</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="2" t="s">
         <v>216</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="D3" s="2" t="s">
         <v>217</v>
       </c>
-      <c r="E3" s="15" t="s">
+      <c r="E3" s="10" t="s">
         <v>218</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A4" s="16" t="s">
+      <c r="A4" s="11" t="s">
         <v>219</v>
       </c>
-      <c r="B4" s="17" t="s">
+      <c r="B4" s="12" t="s">
         <v>220</v>
       </c>
-      <c r="C4" s="17" t="s">
+      <c r="C4" s="12" t="s">
         <v>221</v>
       </c>
-      <c r="D4" s="17" t="s">
+      <c r="D4" s="12" t="s">
         <v>222</v>
       </c>
-      <c r="E4" s="18" t="s">
+      <c r="E4" s="13" t="s">
         <v>223</v>
       </c>
     </row>
@@ -3407,138 +3610,138 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="6" t="s">
         <v>224</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="7" t="s">
         <v>225</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" s="7" t="s">
         <v>226</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="D1" s="7" t="s">
         <v>227</v>
       </c>
-      <c r="E1" s="13" t="s">
+      <c r="E1" s="8" t="s">
         <v>228</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="9" t="s">
         <v>229</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="2" t="s">
         <v>230</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="C2" s="2" t="s">
         <v>231</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="D2" s="2" t="s">
         <v>232</v>
       </c>
-      <c r="E2" s="15" t="s">
+      <c r="E2" s="10" t="s">
         <v>233</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="14" t="s">
+      <c r="A3" s="9" t="s">
         <v>234</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="2" t="s">
         <v>235</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="2" t="s">
         <v>236</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="D3" s="2" t="s">
         <v>237</v>
       </c>
-      <c r="E3" s="15" t="s">
+      <c r="E3" s="10" t="s">
         <v>238</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A4" s="14" t="s">
+      <c r="A4" s="9" t="s">
         <v>239</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="2" t="s">
         <v>241</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="D4" s="2" t="s">
         <v>242</v>
       </c>
-      <c r="E4" s="15" t="s">
+      <c r="E4" s="10" t="s">
         <v>243</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="14" t="s">
+      <c r="A5" s="9" t="s">
         <v>244</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="2" t="s">
         <v>245</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="2" t="s">
         <v>246</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="D5" s="2" t="s">
         <v>247</v>
       </c>
-      <c r="E5" s="15" t="s">
+      <c r="E5" s="10" t="s">
         <v>248</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="14" t="s">
+      <c r="A6" s="9" t="s">
         <v>249</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="2" t="s">
         <v>250</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="2" t="s">
         <v>251</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="2" t="s">
         <v>252</v>
       </c>
-      <c r="E6" s="15" t="s">
+      <c r="E6" s="10" t="s">
         <v>253</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="14" t="s">
+      <c r="A7" s="9" t="s">
         <v>254</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="2" t="s">
         <v>255</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="2" t="s">
         <v>256</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="D7" s="2" t="s">
         <v>257</v>
       </c>
-      <c r="E7" s="15" t="s">
+      <c r="E7" s="10" t="s">
         <v>258</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="16" t="s">
+      <c r="A8" s="11" t="s">
         <v>259</v>
       </c>
-      <c r="B8" s="17" t="s">
+      <c r="B8" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="C8" s="17" t="s">
+      <c r="C8" s="12" t="s">
         <v>260</v>
       </c>
-      <c r="D8" s="17" t="s">
+      <c r="D8" s="12" t="s">
         <v>261</v>
       </c>
-      <c r="E8" s="18" t="s">
+      <c r="E8" s="13" t="s">
         <v>262</v>
       </c>
     </row>
@@ -3565,68 +3768,68 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="6" t="s">
         <v>263</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="7" t="s">
         <v>264</v>
       </c>
-      <c r="C1" s="13" t="s">
+      <c r="C1" s="8" t="s">
         <v>265</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="9" t="s">
         <v>266</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="2" t="s">
         <v>267</v>
       </c>
-      <c r="C2" s="15" t="s">
+      <c r="C2" s="10" t="s">
         <v>268</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="14" t="s">
+      <c r="A3" s="9" t="s">
         <v>269</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="2" t="s">
         <v>270</v>
       </c>
-      <c r="C3" s="15" t="s">
+      <c r="C3" s="10" t="s">
         <v>271</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="14" t="s">
+      <c r="A4" s="9" t="s">
         <v>272</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="2" t="s">
         <v>273</v>
       </c>
-      <c r="C4" s="15" t="s">
+      <c r="C4" s="10" t="s">
         <v>274</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="14" t="s">
+      <c r="A5" s="9" t="s">
         <v>275</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="C5" s="15" t="s">
+      <c r="C5" s="10" t="s">
         <v>277</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="16" t="s">
+      <c r="A6" s="11" t="s">
         <v>278</v>
       </c>
-      <c r="B6" s="17" t="s">
+      <c r="B6" s="12" t="s">
         <v>279</v>
       </c>
-      <c r="C6" s="18" t="s">
+      <c r="C6" s="13" t="s">
         <v>280</v>
       </c>
     </row>
@@ -3639,6 +3842,105 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B885AB6-0F73-44E7-9526-4042DE7247CB}">
+  <dimension ref="B3:J9"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="9.140625" style="22"/>
+    <col min="2" max="2" width="15.85546875" style="22" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="61" style="22" bestFit="1" customWidth="1"/>
+    <col min="4" max="8" width="9.140625" style="22"/>
+    <col min="9" max="9" width="14.140625" style="22" customWidth="1"/>
+    <col min="10" max="10" width="39.7109375" style="22" bestFit="1" customWidth="1"/>
+    <col min="11" max="16384" width="9.140625" style="22"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B3" s="26" t="s">
+        <v>297</v>
+      </c>
+      <c r="C3" s="26"/>
+      <c r="D3" s="26"/>
+      <c r="E3" s="26"/>
+      <c r="F3" s="26"/>
+      <c r="G3" s="26"/>
+      <c r="H3" s="26"/>
+      <c r="I3" s="26"/>
+      <c r="J3" s="26"/>
+    </row>
+    <row r="5" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B5" s="24" t="s">
+        <v>281</v>
+      </c>
+      <c r="C5" s="21" t="s">
+        <v>282</v>
+      </c>
+      <c r="G5" s="25" t="s">
+        <v>290</v>
+      </c>
+      <c r="H5" s="21" t="s">
+        <v>294</v>
+      </c>
+      <c r="I5" s="25" t="s">
+        <v>292</v>
+      </c>
+      <c r="J5" s="21" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="6" spans="2:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="B6" s="24" t="s">
+        <v>283</v>
+      </c>
+      <c r="C6" s="23" t="s">
+        <v>284</v>
+      </c>
+      <c r="G6" s="25" t="s">
+        <v>291</v>
+      </c>
+      <c r="H6" s="21" t="s">
+        <v>27</v>
+      </c>
+      <c r="I6" s="25" t="s">
+        <v>293</v>
+      </c>
+      <c r="J6" s="21" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="2:10" ht="330" x14ac:dyDescent="0.25">
+      <c r="B7" s="24" t="s">
+        <v>285</v>
+      </c>
+      <c r="C7" s="23" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="8" spans="2:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="B8" s="24" t="s">
+        <v>286</v>
+      </c>
+      <c r="C8" s="23" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="9" spans="2:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="B9" s="24" t="s">
+        <v>287</v>
+      </c>
+      <c r="C9" s="23" t="s">
+        <v>288</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B3:J3"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{c5527f93-5752-403e-80d1-f2a7f7fe2faa}" enabled="1" method="Standard" siteId="{9034c6bc-4c08-4727-b3e7-ec2b28440742}" removed="0"/>

</xml_diff>

<commit_message>
Update Framework Proposal and Patient Inbox test plan
</commit_message>
<xml_diff>
--- a/docs/US42595_Patient_Inbox_Email_Multiple_Items_Test_Plan_AC_Traceability.xlsx
+++ b/docs/US42595_Patient_Inbox_Email_Multiple_Items_Test_Plan_AC_Traceability.xlsx
@@ -8,27 +8,25 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://fidelitylifenz-my.sharepoint.com/personal/deepika_udesh_fidelitylife_co_nz/Documents/Desktop/NotepadProject/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="67" documentId="8_{C2FB42C4-CAD5-4EC6-8FCC-E4D329301FD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CEF4C77F-334B-451D-B34C-896186627017}"/>
+  <xr:revisionPtr revIDLastSave="88" documentId="8_{C2FB42C4-CAD5-4EC6-8FCC-E4D329301FD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AF5B05E4-9110-496B-AFCC-0B5C025A2394}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
     <sheet name="Test Cases" sheetId="2" r:id="rId2"/>
-    <sheet name="AC Traceability" sheetId="3" r:id="rId3"/>
-    <sheet name="Risk Areas" sheetId="4" r:id="rId4"/>
-    <sheet name="Test Data" sheetId="5" r:id="rId5"/>
-    <sheet name="Out of Scope" sheetId="6" r:id="rId6"/>
-    <sheet name="Defect Report" sheetId="7" r:id="rId7"/>
+    <sheet name="Risk Areas" sheetId="4" r:id="rId3"/>
+    <sheet name="Test Data" sheetId="5" r:id="rId4"/>
+    <sheet name="Out of Scope" sheetId="6" r:id="rId5"/>
+    <sheet name="Defect Report" sheetId="7" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Cases'!$A$1:$K$17</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="2">'AC Traceability'!$1:$1</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="5">'Out of Scope'!$1:$1</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="3">'Risk Areas'!$1:$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Cases'!$A$1:$J$17</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="4">'Out of Scope'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="2">'Risk Areas'!$1:$1</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">Summary!$1:$1</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Test Cases'!$1:$1</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="4">'Test Data'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="3">'Test Data'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -48,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="414" uniqueCount="298">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="244">
   <si>
     <t>Manual Test Plan - User Story 42595: Patient Inbox Email Multiple Items</t>
   </si>
@@ -71,9 +69,6 @@
     <t>Manual risk-aware coverage for PDF conversion, email generation, recipient accuracy, confirmation/cancel paths and Admin Notes.</t>
   </si>
   <si>
-    <t>Surfaces Covered</t>
-  </si>
-  <si>
     <t>Patient Inbox toolbar, Patient Inbox widget toolbar, and Patient Manager Patient Inbox toolbar.</t>
   </si>
   <si>
@@ -102,9 +97,6 @@
   </si>
   <si>
     <t>Type</t>
-  </si>
-  <si>
-    <t>Surface / Mode</t>
   </si>
   <si>
     <t>Acceptance Criteria Covered</t>
@@ -137,9 +129,6 @@
   </si>
   <si>
     <t>Positive</t>
-  </si>
-  <si>
-    <t>Patient Inbox toolbar</t>
   </si>
   <si>
     <t>AC01, AC23</t>
@@ -166,9 +155,6 @@
     <t>Buttons are displayed in required toolbar locations with correct order and standard UI behaviour.</t>
   </si>
   <si>
-    <t>Widget, Patient Manager</t>
-  </si>
-  <si>
     <t>AC02, AC03, AC23</t>
   </si>
   <si>
@@ -198,9 +184,6 @@
     <t>Negative</t>
   </si>
   <si>
-    <t>All surfaces</t>
-  </si>
-  <si>
     <t>AC04</t>
   </si>
   <si>
@@ -248,9 +231,6 @@
   </si>
   <si>
     <t>Popup shows correct document count, patient name and patient email with Yes and No buttons.</t>
-  </si>
-  <si>
-    <t>Local client or SMTP</t>
   </si>
   <si>
     <t>AC06</t>
@@ -402,9 +382,6 @@
     <t>Admin Note added with date, staff, recipient, email and item details. Long text truncated in list and full details shown when opened.</t>
   </si>
   <si>
-    <t>Patient record</t>
-  </si>
-  <si>
     <t>AC12, AC22</t>
   </si>
   <si>
@@ -486,9 +463,6 @@
     <t>Both configurations follow same recipient, subject, attachment and Admin Note rules.</t>
   </si>
   <si>
-    <t>Local client, SMTP</t>
-  </si>
-  <si>
     <t>Both modes in scope.</t>
   </si>
   <si>
@@ -543,159 +517,6 @@
     <t>Focused cancellation test for AC18.</t>
   </si>
   <si>
-    <t>AC ID</t>
-  </si>
-  <si>
-    <t>Acceptance Criteria</t>
-  </si>
-  <si>
-    <t>Mapped Test Cases</t>
-  </si>
-  <si>
-    <t>Coverage Status</t>
-  </si>
-  <si>
-    <t>Coverage Notes</t>
-  </si>
-  <si>
-    <t>AC01</t>
-  </si>
-  <si>
-    <t>Two new buttons Email Patient and Email Recipient are added to Patient Inbox Toolbar in the Others section.</t>
-  </si>
-  <si>
-    <t>Covered</t>
-  </si>
-  <si>
-    <t>Mapped to test cases that directly validate this acceptance criterion.</t>
-  </si>
-  <si>
-    <t>AC02</t>
-  </si>
-  <si>
-    <t>When Patient Inbox is used as part of a widget, Email Patient and Email Recipient buttons are on the toolbar in the correct position.</t>
-  </si>
-  <si>
-    <t>AC03</t>
-  </si>
-  <si>
-    <t>When Patient Inbox is opened in Patient Manager, Email Patient and Email Recipient buttons are on the toolbar in the correct position.</t>
-  </si>
-  <si>
-    <t>If no items are ticked in Patient Inbox Grid, Email Patient and Email Recipient buttons cannot be clicked.</t>
-  </si>
-  <si>
-    <t>If patient has no email address in Patient Register, Email Patient button cannot be clicked.</t>
-  </si>
-  <si>
-    <t>If user selects one or multiple items and clicks Email Patient, confirmation popup is displayed.</t>
-  </si>
-  <si>
-    <t>AC07</t>
-  </si>
-  <si>
-    <t>If user clicks Yes on Email Patient confirmation, ticked Inbox items are converted to PDF and attached to a new email using correct screen elements.</t>
-  </si>
-  <si>
-    <t>TC-42595-006, TC-42595-013, TC-42595-014</t>
-  </si>
-  <si>
-    <t>If user clicks No on Email Patient confirmation, popup closes and Patient Inbox is displayed.</t>
-  </si>
-  <si>
-    <t>AC09</t>
-  </si>
-  <si>
-    <t>To email address is the address in Patient Register.</t>
-  </si>
-  <si>
-    <t>AC10</t>
-  </si>
-  <si>
-    <t>Subject in Email Patient email follows the specifications.</t>
-  </si>
-  <si>
-    <t>TC-42595-006, TC-42595-012</t>
-  </si>
-  <si>
-    <t>AC11</t>
-  </si>
-  <si>
-    <t>Attachment file names in Email Patient email follow the specifications.</t>
-  </si>
-  <si>
-    <t>AC12</t>
-  </si>
-  <si>
-    <t>Admin Note has been added according to the specifications for Email Patient.</t>
-  </si>
-  <si>
-    <t>If user selects one or multiple items and clicks Email Recipient, search Address Book window is displayed.</t>
-  </si>
-  <si>
-    <t>AC14</t>
-  </si>
-  <si>
-    <t>If user selects a contact with no email recorded, the warning is displayed.</t>
-  </si>
-  <si>
-    <t>AC15</t>
-  </si>
-  <si>
-    <t>If user clicks OK on warning, popup is closed and search Address Book window is displayed.</t>
-  </si>
-  <si>
-    <t>AC16</t>
-  </si>
-  <si>
-    <t>If user selects contact with an email address recorded, email confirmation popup is displayed.</t>
-  </si>
-  <si>
-    <t>AC17</t>
-  </si>
-  <si>
-    <t>If user clicks Yes on To Recipient confirmation, ticked Inbox items are converted to PDF and attached to a new email using correct screen elements.</t>
-  </si>
-  <si>
-    <t>TC-42595-010, TC-42595-013, TC-42595-014</t>
-  </si>
-  <si>
-    <t>If user clicks No on To Recipient confirmation, popup closes and Address Book is displayed.</t>
-  </si>
-  <si>
-    <t>AC19</t>
-  </si>
-  <si>
-    <t>To email address is the address for the contact in Address Book.</t>
-  </si>
-  <si>
-    <t>AC20</t>
-  </si>
-  <si>
-    <t>Subject in To Recipient email follows the specifications.</t>
-  </si>
-  <si>
-    <t>TC-42595-010, TC-42595-012</t>
-  </si>
-  <si>
-    <t>AC21</t>
-  </si>
-  <si>
-    <t>Attachment file names in To Recipient email follow the specifications.</t>
-  </si>
-  <si>
-    <t>AC22</t>
-  </si>
-  <si>
-    <t>Admin Note has been added according to the specifications for To Recipient.</t>
-  </si>
-  <si>
-    <t>All panels, fonts and controls follow Medtech Evolution standards and guidelines.</t>
-  </si>
-  <si>
-    <t>TC-42595-001, TC-42595-002, TC-42595-015</t>
-  </si>
-  <si>
     <t>Risk ID</t>
   </si>
   <si>
@@ -934,9 +755,6 @@
   </si>
   <si>
     <t>Description:</t>
-  </si>
-  <si>
-    <t>The Email Patient button is not displayed in the Others section of the Patient Inbox toolbar. The Email Recipient button is visible, but the Email Patient button is missing.</t>
   </si>
   <si>
     <t>Repro Steps:</t>
@@ -971,6 +789,12 @@
   </si>
   <si>
     <t>42595 - Patient Inbox: Email Multiple Items</t>
+  </si>
+  <si>
+    <t>Sample Defect Report</t>
+  </si>
+  <si>
+    <t>Areas Covered</t>
   </si>
   <si>
     <r>
@@ -982,7 +806,30 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve">PreConditions: </t>
+      <t xml:space="preserve">Env: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">UAT
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">TestData: &lt;&lt;Patient Record Used&gt;&gt;
+PreConditions: </t>
     </r>
     <r>
       <rPr>
@@ -1032,7 +879,8 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>AC Impacted:</t>
+      <t xml:space="preserve">
+AC Impacted:</t>
     </r>
     <r>
       <rPr>
@@ -1094,7 +942,19 @@
     </r>
   </si>
   <si>
-    <t>Sample Defect Report</t>
+    <t>Assignee:</t>
+  </si>
+  <si>
+    <t>XXXXXX</t>
+  </si>
+  <si>
+    <t>Status:</t>
+  </si>
+  <si>
+    <t>New</t>
+  </si>
+  <si>
+    <t>The "Email Patient" button is not displayed in the Others section of the Patient Inbox toolbar. The "Email Recipient" button is visible, but the "Email Patient" button is missing.</t>
   </si>
 </sst>
 </file>
@@ -1330,7 +1190,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1341,9 +1201,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1402,7 +1259,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="32">
+  <dxfs count="25">
     <dxf>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
@@ -1827,141 +1684,6 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
       </border>
     </dxf>
     <dxf>
@@ -2003,20 +1725,6 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="ACTraceabilityTable" displayName="ACTraceabilityTable" ref="A1:E24" headerRowDxfId="31" headerRowBorderDxfId="30">
-  <autoFilter ref="A1:E24" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
-  <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="AC ID" dataDxfId="29"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Acceptance Criteria" dataDxfId="28"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Mapped Test Cases" dataDxfId="27"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Coverage Status" dataDxfId="26"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Coverage Notes" dataDxfId="25"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="RiskAreasTable" displayName="RiskAreasTable" ref="A1:E4" headerRowDxfId="24" totalsRowDxfId="21" headerRowBorderDxfId="23" tableBorderDxfId="22">
   <autoFilter ref="A1:E4" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
   <tableColumns count="5">
@@ -2030,7 +1738,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="TestDataTable" displayName="TestDataTable" ref="A1:E8" headerRowDxfId="15" totalsRowDxfId="12" headerRowBorderDxfId="14" tableBorderDxfId="13">
   <autoFilter ref="A1:E8" xr:uid="{00000000-0009-0000-0100-000003000000}"/>
   <tableColumns count="5">
@@ -2044,7 +1752,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="OutofScopeTable" displayName="OutofScopeTable" ref="A1:C6" headerRowDxfId="6" totalsRowDxfId="3" headerRowBorderDxfId="5" tableBorderDxfId="4">
   <autoFilter ref="A1:C6" xr:uid="{00000000-0009-0000-0100-000004000000}"/>
   <tableColumns count="3">
@@ -2353,81 +2061,81 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="19"/>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
-      <c r="E1" s="19"/>
-      <c r="F1" s="19"/>
-      <c r="G1" s="19"/>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="18"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="16" t="s">
+      <c r="B2" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
-      <c r="G2" s="17"/>
+      <c r="C2" s="16"/>
+      <c r="D2" s="16"/>
+      <c r="E2" s="16"/>
+      <c r="F2" s="16"/>
+      <c r="G2" s="16"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="16" t="s">
+      <c r="B3" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="17"/>
-      <c r="D3" s="17"/>
-      <c r="E3" s="17"/>
-      <c r="F3" s="17"/>
-      <c r="G3" s="17"/>
+      <c r="C3" s="16"/>
+      <c r="D3" s="16"/>
+      <c r="E3" s="16"/>
+      <c r="F3" s="16"/>
+      <c r="G3" s="16"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="16" t="s">
+      <c r="B4" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="17"/>
-      <c r="D4" s="17"/>
-      <c r="E4" s="17"/>
-      <c r="F4" s="17"/>
-      <c r="G4" s="17"/>
+      <c r="C4" s="16"/>
+      <c r="D4" s="16"/>
+      <c r="E4" s="16"/>
+      <c r="F4" s="16"/>
+      <c r="G4" s="16"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="B5" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="16" t="s">
-        <v>8</v>
-      </c>
-      <c r="C5" s="17"/>
-      <c r="D5" s="17"/>
-      <c r="E5" s="17"/>
-      <c r="F5" s="17"/>
-      <c r="G5" s="17"/>
+      <c r="C5" s="16"/>
+      <c r="D5" s="16"/>
+      <c r="E5" s="16"/>
+      <c r="F5" s="16"/>
+      <c r="G5" s="16"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" s="20" t="str">
-        <f>COUNTIF('AC Traceability'!D:D,"Covered")&amp;" of "&amp;COUNTA('AC Traceability'!A:A)-1&amp;" covered"</f>
-        <v>23 of 23 covered</v>
-      </c>
-      <c r="C6" s="17"/>
-      <c r="D6" s="17"/>
-      <c r="E6" s="17"/>
-      <c r="F6" s="17"/>
-      <c r="G6" s="17"/>
+        <v>8</v>
+      </c>
+      <c r="B6" s="19" t="e">
+        <f>COUNTIF(#REF!,"Covered")&amp;" of "&amp;COUNTA(#REF!)-1&amp;" covered"</f>
+        <v>#REF!</v>
+      </c>
+      <c r="C6" s="16"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="16"/>
+      <c r="F6" s="16"/>
+      <c r="G6" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -2448,7 +2156,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K17"/>
+  <dimension ref="A1:J17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -2458,608 +2166,556 @@
     <col min="6" max="6" width="55" customWidth="1"/>
     <col min="7" max="7" width="10" customWidth="1"/>
     <col min="8" max="8" width="14" customWidth="1"/>
-    <col min="9" max="9" width="20" customWidth="1"/>
-    <col min="10" max="10" width="28" customWidth="1"/>
-    <col min="11" max="11" width="32" customWidth="1"/>
+    <col min="9" max="9" width="28" customWidth="1"/>
+    <col min="10" max="10" width="32" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="C1" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="D1" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="E1" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="F1" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="G1" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="H1" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="I1" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="J1" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="J1" s="4" t="s">
+    </row>
+    <row r="2" spans="1:10" ht="87.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="B2" s="2" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" ht="87.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="G2" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="H2" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="G2" s="14" t="s">
+      <c r="I2" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="J2" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="I2" s="2" t="s">
+    </row>
+    <row r="3" spans="1:10" ht="87.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="J2" s="3" t="s">
+      <c r="B3" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="K2" s="2" t="s">
+      <c r="D3" s="2" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="3" spans="1:11" ht="87.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C3" s="2" t="s">
+      <c r="F3" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="G3" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="I3" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="J3" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="F3" s="2" t="s">
+    </row>
+    <row r="4" spans="1:10" ht="87.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="G3" s="14" t="s">
-        <v>27</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="I3" s="2" t="s">
+      <c r="B4" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="J3" s="3" t="s">
+      <c r="C4" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="K3" s="2" t="s">
+      <c r="D4" s="2" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="4" spans="1:11" ht="87.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
+      <c r="E4" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="F4" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="G4" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="H4" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="I4" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="J4" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="F4" s="2" t="s">
+    </row>
+    <row r="5" spans="1:10" ht="87.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="G4" s="14" t="s">
-        <v>27</v>
-      </c>
-      <c r="H4" s="2" t="s">
+      <c r="B5" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="I4" s="2" t="s">
+      <c r="D5" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="J4" s="3" t="s">
+      <c r="E5" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="K4" s="2" t="s">
+      <c r="F5" s="2" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="5" spans="1:11" ht="87.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
+      <c r="G5" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="I5" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="C5" s="2" t="s">
+      <c r="J5" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="D5" s="2" t="s">
+    </row>
+    <row r="6" spans="1:10" ht="87.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="B6" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="C6" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="G5" s="14" t="s">
-        <v>27</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="I5" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="J5" s="3" t="s">
+      <c r="D6" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="K5" s="2" t="s">
+      <c r="E6" s="2" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="6" spans="1:11" ht="87.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
+      <c r="F6" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="G6" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="I6" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="J6" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D6" s="2" t="s">
+    </row>
+    <row r="7" spans="1:10" ht="87.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="B7" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="F6" s="2" t="s">
+      <c r="D7" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="G6" s="14" t="s">
-        <v>27</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="I6" s="2" t="s">
+      <c r="E7" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="J6" s="3" t="s">
+      <c r="F7" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="K6" s="2" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" ht="87.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
+      <c r="G7" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="I7" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="B7" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="C7" s="2" t="s">
+      <c r="J7" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="D7" s="2" t="s">
+    </row>
+    <row r="8" spans="1:10" ht="87.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="B8" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="F7" s="2" t="s">
+      <c r="D8" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="G7" s="14" t="s">
-        <v>27</v>
-      </c>
-      <c r="H7" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="I7" s="2" t="s">
+      <c r="E8" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="J7" s="3" t="s">
+      <c r="F8" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="K7" s="2" t="s">
+      <c r="G8" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="I8" s="3" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="8" spans="1:11" ht="87.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
+      <c r="J8" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="B8" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="C8" s="2" t="s">
+    </row>
+    <row r="9" spans="1:10" ht="87.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="B9" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="C9" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="D9" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="G8" s="14" t="s">
-        <v>27</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="I8" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="J8" s="3" t="s">
+      <c r="E9" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="K8" s="2" t="s">
+      <c r="F9" s="2" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="9" spans="1:11" ht="87.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
+      <c r="G9" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="I9" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="J9" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="C9" s="2" t="s">
+    </row>
+    <row r="10" spans="1:10" ht="87.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="B10" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="D10" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="F9" s="2" t="s">
+      <c r="E10" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="G9" s="14" t="s">
-        <v>27</v>
-      </c>
-      <c r="H9" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="I9" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="J9" s="3" t="s">
+      <c r="F10" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="K9" s="2" t="s">
+      <c r="G10" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="I10" s="3" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="10" spans="1:11" ht="87.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
+      <c r="J10" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="B10" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="C10" s="2" t="s">
+    </row>
+    <row r="11" spans="1:10" ht="87.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="B11" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="E10" s="2" t="s">
+      <c r="D11" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="F10" s="2" t="s">
+      <c r="E11" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="G10" s="14" t="s">
-        <v>27</v>
-      </c>
-      <c r="H10" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="I10" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="J10" s="3" t="s">
+      <c r="F11" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="K10" s="2" t="s">
+      <c r="G11" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="I11" s="3" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="11" spans="1:11" ht="87.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
+      <c r="J11" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="B11" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="C11" s="2" t="s">
+    </row>
+    <row r="12" spans="1:10" ht="87.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="B12" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="E11" s="2" t="s">
+      <c r="C12" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="F11" s="2" t="s">
+      <c r="D12" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="G11" s="14" t="s">
-        <v>27</v>
-      </c>
-      <c r="H11" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="I11" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="J11" s="3" t="s">
+      <c r="E12" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="K11" s="2" t="s">
+      <c r="F12" s="2" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="12" spans="1:11" ht="87.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
+      <c r="G12" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="I12" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="J12" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="C12" s="2" t="s">
+    </row>
+    <row r="13" spans="1:10" ht="87.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="B13" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="E12" s="2" t="s">
+      <c r="C13" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="F12" s="2" t="s">
+      <c r="D13" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="G12" s="14" t="s">
-        <v>27</v>
-      </c>
-      <c r="H12" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="I12" s="2" t="s">
+      <c r="E13" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="J12" s="3" t="s">
+      <c r="F13" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="K12" s="2" t="s">
+      <c r="G13" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="I13" s="3" t="s">
         <v>111</v>
       </c>
-    </row>
-    <row r="13" spans="1:11" ht="87.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
+      <c r="J13" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="B13" s="2" t="s">
+    </row>
+    <row r="14" spans="1:10" ht="87.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="B14" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="D13" s="2" t="s">
+      <c r="C14" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="E13" s="2" t="s">
+      <c r="D14" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="F13" s="2" t="s">
+      <c r="E14" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="G13" s="14" t="s">
-        <v>27</v>
-      </c>
-      <c r="H13" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="I13" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="J13" s="3" t="s">
+      <c r="F14" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="K13" s="2" t="s">
+      <c r="G14" s="14" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="14" spans="1:11" ht="87.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="2" t="s">
+      <c r="H14" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="I14" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="J14" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="C14" s="2" t="s">
+    </row>
+    <row r="15" spans="1:10" ht="87.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="D14" s="2" t="s">
+      <c r="B15" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="E14" s="2" t="s">
+      <c r="C15" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="F14" s="2" t="s">
+      <c r="D15" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="G14" s="15" t="s">
+      <c r="E15" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="H14" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="I14" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="J14" s="3" t="s">
+      <c r="F15" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="K14" s="2" t="s">
+      <c r="G15" s="14" t="s">
+        <v>119</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="I15" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="J15" s="2" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="87.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="2" t="s">
+    <row r="16" spans="1:10" ht="87.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B16" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="C16" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="D15" s="2" t="s">
+      <c r="D16" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="E15" s="2" t="s">
+      <c r="E16" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="F15" s="2" t="s">
+      <c r="F16" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="G15" s="15" t="s">
-        <v>126</v>
-      </c>
-      <c r="H15" s="2" t="s">
-        <v>130</v>
-      </c>
-      <c r="I15" s="2" t="s">
+      <c r="G16" s="14" t="s">
+        <v>119</v>
+      </c>
+      <c r="H16" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="J15" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="K15" s="2" t="s">
+      <c r="I16" s="3" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="16" spans="1:11" ht="87.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="2" t="s">
+      <c r="J16" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="B16" s="2" t="s">
+    </row>
+    <row r="17" spans="1:10" ht="87.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="B17" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C17" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="D16" s="2" t="s">
+      <c r="D17" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="E16" s="2" t="s">
+      <c r="E17" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="F16" s="2" t="s">
+      <c r="F17" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="G16" s="15" t="s">
-        <v>126</v>
-      </c>
-      <c r="H16" s="2" t="s">
+      <c r="G17" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="I17" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="I16" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="J16" s="3" t="s">
+      <c r="J17" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="K16" s="2" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" ht="87.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>148</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>149</v>
-      </c>
-      <c r="F17" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="G17" s="14" t="s">
-        <v>27</v>
-      </c>
-      <c r="H17" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="I17" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="J17" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="K17" s="2" t="s">
-        <v>152</v>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K17" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <autoFilter ref="A1:J17" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <dataValidations count="1">
     <dataValidation type="list" sqref="G2:G17" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"P1,P2,P3"</formula1>
@@ -3071,438 +2727,6 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <sheetPr>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="A1:E24"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="12" customWidth="1"/>
-    <col min="2" max="2" width="72" customWidth="1"/>
-    <col min="3" max="3" width="42" customWidth="1"/>
-    <col min="4" max="4" width="18" customWidth="1"/>
-    <col min="5" max="5" width="55" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
-        <v>153</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>154</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
-        <v>158</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>159</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="D2" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
-        <v>164</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>166</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>167</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>168</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>170</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>171</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>172</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>174</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
-        <v>175</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
-        <v>178</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>179</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
-        <v>180</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>181</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="D13" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>182</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="D14" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="2" t="s">
-        <v>183</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>184</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="D15" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="D16" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="2" t="s">
-        <v>187</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>188</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="D17" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="2" t="s">
-        <v>189</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>190</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="D18" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="2" t="s">
-        <v>151</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>192</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="D19" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="E19" s="2" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="2" t="s">
-        <v>193</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="D20" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="E20" s="2" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="D21" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="E21" s="2" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="2" t="s">
-        <v>198</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="D22" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="E22" s="2" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="2" t="s">
-        <v>200</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="D23" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="E23" s="2" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>202</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="D24" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="E24" s="2" t="s">
-        <v>161</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup fitToHeight="0" orientation="landscape"/>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -3518,71 +2742,71 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
-        <v>204</v>
-      </c>
-      <c r="B1" s="7" t="s">
-        <v>205</v>
-      </c>
-      <c r="C1" s="7" t="s">
-        <v>206</v>
-      </c>
-      <c r="D1" s="7" t="s">
-        <v>207</v>
-      </c>
-      <c r="E1" s="8" t="s">
-        <v>208</v>
+      <c r="A1" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>149</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A2" s="9" t="s">
-        <v>209</v>
+      <c r="A2" s="8" t="s">
+        <v>150</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>210</v>
+        <v>151</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>211</v>
+        <v>152</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>212</v>
-      </c>
-      <c r="E2" s="10" t="s">
-        <v>213</v>
+        <v>153</v>
+      </c>
+      <c r="E2" s="9" t="s">
+        <v>154</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A3" s="9" t="s">
-        <v>214</v>
+      <c r="A3" s="8" t="s">
+        <v>155</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>215</v>
+        <v>156</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>216</v>
+        <v>157</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>217</v>
-      </c>
-      <c r="E3" s="10" t="s">
-        <v>218</v>
+        <v>158</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>159</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A4" s="11" t="s">
-        <v>219</v>
-      </c>
-      <c r="B4" s="12" t="s">
-        <v>220</v>
-      </c>
-      <c r="C4" s="12" t="s">
-        <v>221</v>
-      </c>
-      <c r="D4" s="12" t="s">
-        <v>222</v>
-      </c>
-      <c r="E4" s="13" t="s">
-        <v>223</v>
+      <c r="A4" s="10" t="s">
+        <v>160</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>161</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>162</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="E4" s="12" t="s">
+        <v>164</v>
       </c>
     </row>
   </sheetData>
@@ -3594,7 +2818,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -3610,139 +2834,139 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
-        <v>224</v>
-      </c>
-      <c r="B1" s="7" t="s">
-        <v>225</v>
-      </c>
-      <c r="C1" s="7" t="s">
-        <v>226</v>
-      </c>
-      <c r="D1" s="7" t="s">
-        <v>227</v>
-      </c>
-      <c r="E1" s="8" t="s">
-        <v>228</v>
+      <c r="A1" s="5" t="s">
+        <v>165</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>166</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>167</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>169</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="9" t="s">
-        <v>229</v>
+      <c r="A2" s="8" t="s">
+        <v>170</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>230</v>
+        <v>171</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>231</v>
+        <v>172</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>232</v>
-      </c>
-      <c r="E2" s="10" t="s">
-        <v>233</v>
+        <v>173</v>
+      </c>
+      <c r="E2" s="9" t="s">
+        <v>174</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="9" t="s">
-        <v>234</v>
+      <c r="A3" s="8" t="s">
+        <v>175</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>235</v>
+        <v>176</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>236</v>
+        <v>177</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>237</v>
-      </c>
-      <c r="E3" s="10" t="s">
-        <v>238</v>
+        <v>178</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>179</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A4" s="9" t="s">
-        <v>239</v>
+      <c r="A4" s="8" t="s">
+        <v>180</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>240</v>
+        <v>181</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>241</v>
+        <v>182</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>242</v>
-      </c>
-      <c r="E4" s="10" t="s">
-        <v>243</v>
+        <v>183</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>184</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="9" t="s">
-        <v>244</v>
+      <c r="A5" s="8" t="s">
+        <v>185</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>245</v>
+        <v>186</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>246</v>
+        <v>187</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>247</v>
-      </c>
-      <c r="E5" s="10" t="s">
-        <v>248</v>
+        <v>188</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>189</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="9" t="s">
-        <v>249</v>
+      <c r="A6" s="8" t="s">
+        <v>190</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>250</v>
+        <v>191</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>251</v>
+        <v>192</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>252</v>
-      </c>
-      <c r="E6" s="10" t="s">
-        <v>253</v>
+        <v>193</v>
+      </c>
+      <c r="E6" s="9" t="s">
+        <v>194</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="9" t="s">
-        <v>254</v>
+      <c r="A7" s="8" t="s">
+        <v>195</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>255</v>
+        <v>196</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>256</v>
+        <v>197</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>257</v>
-      </c>
-      <c r="E7" s="10" t="s">
-        <v>258</v>
+        <v>198</v>
+      </c>
+      <c r="E7" s="9" t="s">
+        <v>199</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="11" t="s">
-        <v>259</v>
-      </c>
-      <c r="B8" s="12" t="s">
-        <v>71</v>
-      </c>
-      <c r="C8" s="12" t="s">
-        <v>260</v>
-      </c>
-      <c r="D8" s="12" t="s">
-        <v>261</v>
-      </c>
-      <c r="E8" s="13" t="s">
-        <v>262</v>
+      <c r="A8" s="10" t="s">
+        <v>200</v>
+      </c>
+      <c r="B8" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>201</v>
+      </c>
+      <c r="D8" s="11" t="s">
+        <v>202</v>
+      </c>
+      <c r="E8" s="12" t="s">
+        <v>203</v>
       </c>
     </row>
   </sheetData>
@@ -3754,7 +2978,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -3768,69 +2992,69 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
-        <v>263</v>
-      </c>
-      <c r="B1" s="7" t="s">
-        <v>264</v>
-      </c>
-      <c r="C1" s="8" t="s">
-        <v>265</v>
+      <c r="A1" s="5" t="s">
+        <v>204</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>205</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A2" s="9" t="s">
-        <v>266</v>
+      <c r="A2" s="8" t="s">
+        <v>207</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>267</v>
-      </c>
-      <c r="C2" s="10" t="s">
-        <v>268</v>
+        <v>208</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>209</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="9" t="s">
-        <v>269</v>
+      <c r="A3" s="8" t="s">
+        <v>210</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>270</v>
-      </c>
-      <c r="C3" s="10" t="s">
-        <v>271</v>
+        <v>211</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>212</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="9" t="s">
-        <v>272</v>
+      <c r="A4" s="8" t="s">
+        <v>213</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>273</v>
-      </c>
-      <c r="C4" s="10" t="s">
-        <v>274</v>
+        <v>214</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>215</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="9" t="s">
-        <v>275</v>
+      <c r="A5" s="8" t="s">
+        <v>216</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>276</v>
-      </c>
-      <c r="C5" s="10" t="s">
-        <v>277</v>
+        <v>217</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>218</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="11" t="s">
-        <v>278</v>
-      </c>
-      <c r="B6" s="12" t="s">
-        <v>279</v>
-      </c>
-      <c r="C6" s="13" t="s">
-        <v>280</v>
+      <c r="A6" s="10" t="s">
+        <v>219</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>220</v>
+      </c>
+      <c r="C6" s="12" t="s">
+        <v>221</v>
       </c>
     </row>
   </sheetData>
@@ -3842,100 +3066,115 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B885AB6-0F73-44E7-9526-4042DE7247CB}">
-  <dimension ref="B3:J9"/>
+  <dimension ref="B2:L9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.140625" style="22"/>
-    <col min="2" max="2" width="15.85546875" style="22" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="61" style="22" bestFit="1" customWidth="1"/>
-    <col min="4" max="8" width="9.140625" style="22"/>
-    <col min="9" max="9" width="14.140625" style="22" customWidth="1"/>
-    <col min="10" max="10" width="39.7109375" style="22" bestFit="1" customWidth="1"/>
-    <col min="11" max="16384" width="9.140625" style="22"/>
+    <col min="1" max="1" width="9.140625" style="21"/>
+    <col min="2" max="2" width="15.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="61" style="21" bestFit="1" customWidth="1"/>
+    <col min="4" max="8" width="9.140625" style="21"/>
+    <col min="9" max="9" width="14.140625" style="21" customWidth="1"/>
+    <col min="10" max="10" width="39.7109375" style="21" bestFit="1" customWidth="1"/>
+    <col min="11" max="16384" width="9.140625" style="21"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B3" s="26" t="s">
-        <v>297</v>
-      </c>
-      <c r="C3" s="26"/>
-      <c r="D3" s="26"/>
-      <c r="E3" s="26"/>
-      <c r="F3" s="26"/>
-      <c r="G3" s="26"/>
-      <c r="H3" s="26"/>
-      <c r="I3" s="26"/>
-      <c r="J3" s="26"/>
-    </row>
-    <row r="5" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B5" s="24" t="s">
-        <v>281</v>
-      </c>
-      <c r="C5" s="21" t="s">
-        <v>282</v>
-      </c>
-      <c r="G5" s="25" t="s">
-        <v>290</v>
-      </c>
-      <c r="H5" s="21" t="s">
-        <v>294</v>
-      </c>
-      <c r="I5" s="25" t="s">
-        <v>292</v>
-      </c>
-      <c r="J5" s="21" t="s">
-        <v>295</v>
-      </c>
-    </row>
-    <row r="6" spans="2:10" ht="45" x14ac:dyDescent="0.25">
-      <c r="B6" s="24" t="s">
-        <v>283</v>
-      </c>
-      <c r="C6" s="23" t="s">
-        <v>284</v>
-      </c>
-      <c r="G6" s="25" t="s">
-        <v>291</v>
-      </c>
-      <c r="H6" s="21" t="s">
-        <v>27</v>
-      </c>
-      <c r="I6" s="25" t="s">
-        <v>293</v>
-      </c>
-      <c r="J6" s="21" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="7" spans="2:10" ht="330" x14ac:dyDescent="0.25">
-      <c r="B7" s="24" t="s">
-        <v>285</v>
-      </c>
-      <c r="C7" s="23" t="s">
-        <v>296</v>
-      </c>
-    </row>
-    <row r="8" spans="2:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="B8" s="24" t="s">
-        <v>286</v>
-      </c>
-      <c r="C8" s="23" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="9" spans="2:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="B9" s="24" t="s">
-        <v>287</v>
-      </c>
-      <c r="C9" s="23" t="s">
-        <v>288</v>
+    <row r="2" spans="2:12" ht="3.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="3" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B3" s="25" t="s">
+        <v>236</v>
+      </c>
+      <c r="C3" s="25"/>
+      <c r="D3" s="25"/>
+      <c r="E3" s="25"/>
+      <c r="F3" s="25"/>
+      <c r="G3" s="25"/>
+      <c r="H3" s="25"/>
+      <c r="I3" s="25"/>
+      <c r="J3" s="25"/>
+      <c r="K3" s="25"/>
+      <c r="L3" s="25"/>
+    </row>
+    <row r="5" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B5" s="23" t="s">
+        <v>222</v>
+      </c>
+      <c r="C5" s="20" t="s">
+        <v>223</v>
+      </c>
+      <c r="G5" s="24" t="s">
+        <v>230</v>
+      </c>
+      <c r="H5" s="20" t="s">
+        <v>234</v>
+      </c>
+      <c r="I5" s="24" t="s">
+        <v>232</v>
+      </c>
+      <c r="J5" s="20" t="s">
+        <v>235</v>
+      </c>
+      <c r="K5" s="24" t="s">
+        <v>239</v>
+      </c>
+      <c r="L5" s="20" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="6" spans="2:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="B6" s="23" t="s">
+        <v>224</v>
+      </c>
+      <c r="C6" s="22" t="s">
+        <v>243</v>
+      </c>
+      <c r="G6" s="24" t="s">
+        <v>231</v>
+      </c>
+      <c r="H6" s="20" t="s">
+        <v>25</v>
+      </c>
+      <c r="I6" s="24" t="s">
+        <v>233</v>
+      </c>
+      <c r="J6" s="20" t="s">
+        <v>19</v>
+      </c>
+      <c r="K6" s="24" t="s">
+        <v>241</v>
+      </c>
+      <c r="L6" s="20" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="7" spans="2:12" ht="360" x14ac:dyDescent="0.25">
+      <c r="B7" s="23" t="s">
+        <v>225</v>
+      </c>
+      <c r="C7" s="22" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="8" spans="2:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="B8" s="23" t="s">
+        <v>226</v>
+      </c>
+      <c r="C8" s="22" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="9" spans="2:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="B9" s="23" t="s">
+        <v>227</v>
+      </c>
+      <c r="C9" s="22" t="s">
+        <v>228</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="B3:J3"/>
+    <mergeCell ref="B3:L3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>